<commit_message>
Aplica o período letivo real do 1º semestre: 04/02 a 10/07
A escola confirmou as datas. Antes o cálculo contava semanas inteiras a
partir da semana 1 do Klausurplan (02/02), o que incluía indevidamente a
segunda e a terça anteriores ao início das aulas. Agora cada (semana,
dia) é convertido em data e comparado com o período letivo, além de
continuar descontando os dias marcados como 'unterrichtsfrei'.

Efeito: duas aulas a menos por slot de segunda e terça. Ex.: Matemática
da 9C1 passa de 105 para 103 aulas no semestre. Os percentuais sobem
levemente — Química/CAl na 12C1 vai de 18,2% para 19,0%.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Comparativo_Cessoes_1SEM_x_Proposta3.xlsx
+++ b/Horario desenvolvido/Comparativo_Cessoes_1SEM_x_Proposta3.xlsx
@@ -576,7 +576,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>0.1818181818181818</v>
+        <v>0.1904761904761905</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>0</v>
@@ -585,7 +585,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>-0.1818181818181818</v>
+        <v>-0.1904761904761905</v>
       </c>
     </row>
     <row r="5">
@@ -608,7 +608,7 @@
         <v>3</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>0.1363636363636364</v>
+        <v>0.1428571428571428</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>0</v>
@@ -617,7 +617,7 @@
         <v>0</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>-0.1363636363636364</v>
+        <v>-0.1428571428571428</v>
       </c>
     </row>
     <row r="6">
@@ -704,7 +704,7 @@
         <v>2</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>0.09523809523809523</v>
+        <v>0.1</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>0</v>
@@ -713,7 +713,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>-0.09523809523809523</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="9">
@@ -736,7 +736,7 @@
         <v>6</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>0.09375</v>
+        <v>0.09836065573770492</v>
       </c>
       <c r="F9" s="4" t="n">
         <v>0</v>
@@ -745,7 +745,7 @@
         <v>0</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>-0.09375</v>
+        <v>-0.09836065573770492</v>
       </c>
     </row>
     <row r="10">
@@ -768,7 +768,7 @@
         <v>2</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.09523809523809523</v>
       </c>
       <c r="F10" s="4" t="n">
         <v>0</v>
@@ -777,7 +777,7 @@
         <v>0</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>-0.09090909090909091</v>
+        <v>-0.09523809523809523</v>
       </c>
     </row>
     <row r="11">
@@ -800,7 +800,7 @@
         <v>2</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.09523809523809523</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>0</v>
@@ -809,7 +809,7 @@
         <v>0</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>-0.09090909090909091</v>
+        <v>-0.09523809523809523</v>
       </c>
     </row>
     <row r="12">
@@ -911,7 +911,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>10C2</t>
+          <t>10C1</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -928,7 +928,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>0.009708737864077669</v>
+        <v>0.009900990099009901</v>
       </c>
       <c r="F15" s="4" t="n">
         <v>6</v>
@@ -937,13 +937,13 @@
         <v>0.08823529411764706</v>
       </c>
       <c r="H15" s="8" t="n">
-        <v>0.0785265562535694</v>
+        <v>0.07833430401863717</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>10C1</t>
+          <t>10C2</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -960,7 +960,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>0.009708737864077669</v>
+        <v>0.009900990099009901</v>
       </c>
       <c r="F16" s="4" t="n">
         <v>6</v>
@@ -969,7 +969,7 @@
         <v>0.08823529411764706</v>
       </c>
       <c r="H16" s="8" t="n">
-        <v>0.0785265562535694</v>
+        <v>0.07833430401863717</v>
       </c>
     </row>
     <row r="17">
@@ -980,12 +980,12 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Port</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>MFo</t>
+          <t>FBri</t>
         </is>
       </c>
       <c r="D17" s="4" t="n">
@@ -1012,12 +1012,12 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Port</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>FBri</t>
+          <t>MFo</t>
         </is>
       </c>
       <c r="D18" s="4" t="n">
@@ -1071,49 +1071,49 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>10C2</t>
+          <t>11C1</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Hist</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>ALu</t>
+          <t>ClaMe</t>
         </is>
       </c>
       <c r="D20" s="4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>0</v>
+        <v>0.1162790697674419</v>
       </c>
       <c r="F20" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>0.07142857142857142</v>
-      </c>
-      <c r="H20" s="8" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.04347826086956522</v>
+      </c>
+      <c r="H20" s="7" t="n">
+        <v>-0.07280080889787668</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>10C1</t>
+          <t>12C2</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Fis</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>CAl</t>
+          <t>Cadu</t>
         </is>
       </c>
       <c r="D21" s="4" t="n">
@@ -1135,145 +1135,145 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>12C2</t>
+          <t>12C1</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Fis</t>
+          <t>Hist</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Cadu</t>
+          <t>Wag</t>
         </is>
       </c>
       <c r="D22" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>0</v>
+        <v>0.07142857142857142</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>0.07142857142857142</v>
-      </c>
-      <c r="H22" s="8" t="n">
-        <v>0.07142857142857142</v>
+        <v>0</v>
+      </c>
+      <c r="H22" s="7" t="n">
+        <v>-0.07142857142857142</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>11C1</t>
+          <t>10C2</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Hist</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>ClaMe</t>
+          <t>ALu</t>
         </is>
       </c>
       <c r="D23" s="4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>0.1136363636363636</v>
+        <v>0</v>
       </c>
       <c r="F23" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>0.04347826086956522</v>
-      </c>
-      <c r="H23" s="7" t="n">
-        <v>-0.07015810276679837</v>
+        <v>0.07142857142857142</v>
+      </c>
+      <c r="H23" s="8" t="n">
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>12C1</t>
+          <t>10C1</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Hist</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Wag</t>
+          <t>CAl</t>
         </is>
       </c>
       <c r="D24" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>0.06976744186046512</v>
+        <v>0</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="7" t="n">
-        <v>-0.06976744186046512</v>
+        <v>0.07142857142857142</v>
+      </c>
+      <c r="H24" s="8" t="n">
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>11C2</t>
+          <t>9C2</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>GL</t>
+          <t>Hist</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>CBu</t>
+          <t>JuLa</t>
         </is>
       </c>
       <c r="D25" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G25" s="6" t="n">
-        <v>0.06666666666666667</v>
-      </c>
-      <c r="H25" s="8" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.03333333333333333</v>
+      </c>
+      <c r="H25" s="7" t="n">
+        <v>-0.06666666666666668</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>11C1</t>
+          <t>11C2</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Port</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>AMu</t>
+          <t>CBu</t>
         </is>
       </c>
       <c r="D26" s="4" t="n">
@@ -1286,90 +1286,90 @@
         <v>2</v>
       </c>
       <c r="G26" s="6" t="n">
-        <v>0.06451612903225806</v>
+        <v>0.06666666666666667</v>
       </c>
       <c r="H26" s="8" t="n">
-        <v>0.06451612903225806</v>
+        <v>0.06666666666666667</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>12C1</t>
+          <t>11C1</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Geo</t>
+          <t>Port</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>AMu</t>
         </is>
       </c>
       <c r="D27" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>0.01538461538461539</v>
+        <v>0</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>0.07894736842105263</v>
+        <v>0.06451612903225806</v>
       </c>
       <c r="H27" s="8" t="n">
-        <v>0.06356275303643724</v>
+        <v>0.06451612903225806</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>11C1</t>
+          <t>12C1</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Geo</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>JJ</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D28" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>0</v>
+        <v>0.01587301587301587</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>0.0625</v>
+        <v>0.07894736842105263</v>
       </c>
       <c r="H28" s="8" t="n">
-        <v>0.0625</v>
+        <v>0.06307435254803676</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>11C2</t>
+          <t>9C1</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Port</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>CAl</t>
+          <t>Jana</t>
         </is>
       </c>
       <c r="D29" s="4" t="n">
@@ -1391,17 +1391,17 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>9C1</t>
+          <t>11C1</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Port</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Jana</t>
+          <t>JJ</t>
         </is>
       </c>
       <c r="D30" s="4" t="n">
@@ -1455,33 +1455,33 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>9C2</t>
+          <t>11C2</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Hist</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>JuLa</t>
+          <t>CAl</t>
         </is>
       </c>
       <c r="D32" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>0.09523809523809523</v>
+        <v>0</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G32" s="6" t="n">
-        <v>0.03333333333333333</v>
-      </c>
-      <c r="H32" s="7" t="n">
-        <v>-0.0619047619047619</v>
+        <v>0.0625</v>
+      </c>
+      <c r="H32" s="8" t="n">
+        <v>0.0625</v>
       </c>
     </row>
     <row r="33">
@@ -1504,7 +1504,7 @@
         <v>8</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>0.09195402298850575</v>
+        <v>0.09411764705882353</v>
       </c>
       <c r="F33" s="4" t="n">
         <v>2</v>
@@ -1513,7 +1513,7 @@
         <v>0.03571428571428571</v>
       </c>
       <c r="H33" s="7" t="n">
-        <v>-0.05623973727422003</v>
+        <v>-0.05840336134453782</v>
       </c>
     </row>
     <row r="34">
@@ -1568,7 +1568,7 @@
         <v>1</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>0.02439024390243903</v>
+        <v>0.025</v>
       </c>
       <c r="F35" s="4" t="n">
         <v>2</v>
@@ -1577,7 +1577,7 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="H35" s="8" t="n">
-        <v>0.0525328330206379</v>
+        <v>0.05192307692307693</v>
       </c>
     </row>
     <row r="36">
@@ -1647,97 +1647,97 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>12C2</t>
+          <t>10C1</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Fab</t>
+          <t>Lza</t>
         </is>
       </c>
       <c r="D38" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>0.04878048780487805</v>
+        <v>0.1</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G38" s="6" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="H38" s="7" t="n">
-        <v>-0.04878048780487805</v>
+        <v>-0.05</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>12C1</t>
+          <t>12C2</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Bre</t>
+          <t>Fab</t>
         </is>
       </c>
       <c r="D39" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E39" s="6" t="n">
-        <v>0.02272727272727273</v>
+        <v>0.04878048780487805</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G39" s="6" t="n">
-        <v>0.07142857142857142</v>
-      </c>
-      <c r="H39" s="8" t="n">
-        <v>0.04870129870129869</v>
+        <v>0</v>
+      </c>
+      <c r="H39" s="7" t="n">
+        <v>-0.04878048780487805</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>12C1</t>
+          <t>11C1</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Fis</t>
+          <t>Redação</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Cadu</t>
+          <t>ACo</t>
         </is>
       </c>
       <c r="D40" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>0.02272727272727273</v>
+        <v>0.04878048780487805</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G40" s="6" t="n">
-        <v>0.07142857142857142</v>
-      </c>
-      <c r="H40" s="8" t="n">
-        <v>0.04870129870129869</v>
+        <v>0</v>
+      </c>
+      <c r="H40" s="7" t="n">
+        <v>-0.04878048780487805</v>
       </c>
     </row>
     <row r="41">
@@ -1748,12 +1748,12 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Port</t>
+          <t>Fis</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Deb</t>
+          <t>Cadu</t>
         </is>
       </c>
       <c r="D41" s="4" t="n">
@@ -1763,7 +1763,7 @@
         <v>0.02325581395348837</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G41" s="6" t="n">
         <v>0.07142857142857142</v>
@@ -1775,71 +1775,71 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>10C1</t>
+          <t>12C1</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Port</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>BrSa</t>
+          <t>Deb</t>
         </is>
       </c>
       <c r="D42" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E42" s="6" t="n">
-        <v>0</v>
+        <v>0.02325581395348837</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G42" s="6" t="n">
-        <v>0.04761904761904762</v>
+        <v>0.07142857142857142</v>
       </c>
       <c r="H42" s="8" t="n">
-        <v>0.04761904761904762</v>
+        <v>0.04817275747508305</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>12C1</t>
+          <t>10C1</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Fil</t>
+          <t>Fis</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>LAn</t>
+          <t>VSi</t>
         </is>
       </c>
       <c r="D43" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E43" s="6" t="n">
-        <v>0.04761904761904762</v>
+        <v>0.125</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G43" s="6" t="n">
-        <v>0</v>
+        <v>0.07692307692307693</v>
       </c>
       <c r="H43" s="7" t="n">
-        <v>-0.04761904761904762</v>
+        <v>-0.04807692307692307</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>10C2</t>
+          <t>12C1</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
@@ -1849,46 +1849,46 @@
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>BrSa</t>
+          <t>Bre</t>
         </is>
       </c>
       <c r="D44" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E44" s="6" t="n">
-        <v>0</v>
+        <v>0.02352941176470588</v>
       </c>
       <c r="F44" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G44" s="6" t="n">
-        <v>0.04761904761904762</v>
+        <v>0.07142857142857142</v>
       </c>
       <c r="H44" s="8" t="n">
-        <v>0.04761904761904762</v>
+        <v>0.04789915966386554</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>11C2</t>
+          <t>12C1</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Hist</t>
+          <t>Fil</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Ver</t>
+          <t>LAn</t>
         </is>
       </c>
       <c r="D45" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E45" s="6" t="n">
-        <v>0.04651162790697674</v>
+        <v>0.04761904761904762</v>
       </c>
       <c r="F45" s="4" t="n">
         <v>0</v>
@@ -1897,39 +1897,39 @@
         <v>0</v>
       </c>
       <c r="H45" s="7" t="n">
-        <v>-0.04651162790697674</v>
+        <v>-0.04761904761904762</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>11C1</t>
+          <t>10C2</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Redação</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>ACo</t>
+          <t>BrSa</t>
         </is>
       </c>
       <c r="D46" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>0.04651162790697674</v>
+        <v>0</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G46" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" s="7" t="n">
-        <v>-0.04651162790697674</v>
+        <v>0.04761904761904762</v>
+      </c>
+      <c r="H46" s="8" t="n">
+        <v>0.04761904761904762</v>
       </c>
     </row>
     <row r="47">
@@ -1940,51 +1940,51 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Hist</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>ALu</t>
+          <t>BrSa</t>
         </is>
       </c>
       <c r="D47" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E47" s="6" t="n">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="F47" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G47" s="6" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.04761904761904762</v>
       </c>
       <c r="H47" s="8" t="n">
-        <v>0.04642857142857142</v>
+        <v>0.04761904761904762</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>11C1</t>
+          <t>11C2</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Fil</t>
+          <t>Hist</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>LAn</t>
+          <t>Ver</t>
         </is>
       </c>
       <c r="D48" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E48" s="6" t="n">
-        <v>0.04545454545454546</v>
+        <v>0.04761904761904762</v>
       </c>
       <c r="F48" s="4" t="n">
         <v>0</v>
@@ -1993,7 +1993,7 @@
         <v>0</v>
       </c>
       <c r="H48" s="7" t="n">
-        <v>-0.04545454545454546</v>
+        <v>-0.04761904761904762</v>
       </c>
     </row>
     <row r="49">
@@ -2016,7 +2016,7 @@
         <v>2</v>
       </c>
       <c r="E49" s="6" t="n">
-        <v>0.04545454545454546</v>
+        <v>0.04651162790697674</v>
       </c>
       <c r="F49" s="4" t="n">
         <v>0</v>
@@ -2025,7 +2025,7 @@
         <v>0</v>
       </c>
       <c r="H49" s="7" t="n">
-        <v>-0.04545454545454546</v>
+        <v>-0.04651162790697674</v>
       </c>
     </row>
     <row r="50">
@@ -2036,60 +2036,60 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Hist</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Lza</t>
+          <t>ALu</t>
         </is>
       </c>
       <c r="D50" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E50" s="6" t="n">
-        <v>0.09523809523809523</v>
+        <v>0.02564102564102564</v>
       </c>
       <c r="F50" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G50" s="6" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="H50" s="7" t="n">
-        <v>-0.04523809523809523</v>
+        <v>0.07142857142857142</v>
+      </c>
+      <c r="H50" s="8" t="n">
+        <v>0.04578754578754578</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>10C1</t>
+          <t>11C1</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Fis</t>
+          <t>Fil</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>VSi</t>
+          <t>LAn</t>
         </is>
       </c>
       <c r="D51" s="4" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E51" s="6" t="n">
-        <v>0.1219512195121951</v>
+        <v>0.04545454545454546</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G51" s="6" t="n">
-        <v>0.07692307692307693</v>
+        <v>0</v>
       </c>
       <c r="H51" s="7" t="n">
-        <v>-0.04502814258911818</v>
+        <v>-0.04545454545454546</v>
       </c>
     </row>
     <row r="52">
@@ -2127,65 +2127,65 @@
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>12C2</t>
+          <t>11C1</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Port</t>
+          <t>Fis</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
         <is>
-          <t>Deb</t>
+          <t>Cadu</t>
         </is>
       </c>
       <c r="D53" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E53" s="6" t="n">
-        <v>0.06451612903225806</v>
+        <v>0</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G53" s="6" t="n">
-        <v>0.1071428571428571</v>
+        <v>0.04166666666666666</v>
       </c>
       <c r="H53" s="8" t="n">
-        <v>0.04262672811059903</v>
+        <v>0.04166666666666666</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>11C1</t>
+          <t>12C2</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>Fis</t>
+          <t>Port</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Cadu</t>
+          <t>Deb</t>
         </is>
       </c>
       <c r="D54" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E54" s="6" t="n">
-        <v>0</v>
+        <v>0.06557377049180328</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G54" s="6" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.1071428571428571</v>
       </c>
       <c r="H54" s="8" t="n">
-        <v>0.04166666666666666</v>
+        <v>0.04156908665105381</v>
       </c>
     </row>
     <row r="55">
@@ -2208,7 +2208,7 @@
         <v>5</v>
       </c>
       <c r="E55" s="6" t="n">
-        <v>0.08064516129032258</v>
+        <v>0.08196721311475409</v>
       </c>
       <c r="F55" s="4" t="n">
         <v>2</v>
@@ -2217,7 +2217,7 @@
         <v>0.04166666666666666</v>
       </c>
       <c r="H55" s="7" t="n">
-        <v>-0.03897849462365592</v>
+        <v>-0.04030054644808743</v>
       </c>
     </row>
     <row r="56">
@@ -2255,7 +2255,7 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>12C1</t>
+          <t>9C2</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -2265,23 +2265,23 @@
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>PaH</t>
+          <t>APa</t>
         </is>
       </c>
       <c r="D57" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E57" s="6" t="n">
-        <v>0.01538461538461539</v>
+        <v>0.0379746835443038</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G57" s="6" t="n">
-        <v>0.05263157894736842</v>
-      </c>
-      <c r="H57" s="8" t="n">
-        <v>0.03724696356275303</v>
+        <v>0</v>
+      </c>
+      <c r="H57" s="7" t="n">
+        <v>-0.0379746835443038</v>
       </c>
     </row>
     <row r="58">
@@ -2304,7 +2304,7 @@
         <v>3</v>
       </c>
       <c r="E58" s="6" t="n">
-        <v>0.03703703703703703</v>
+        <v>0.0379746835443038</v>
       </c>
       <c r="F58" s="4" t="n">
         <v>0</v>
@@ -2313,13 +2313,13 @@
         <v>0</v>
       </c>
       <c r="H58" s="7" t="n">
-        <v>-0.03703703703703703</v>
+        <v>-0.0379746835443038</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>9C2</t>
+          <t>12C1</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
@@ -2329,39 +2329,39 @@
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>APa</t>
+          <t>PaH</t>
         </is>
       </c>
       <c r="D59" s="4" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E59" s="6" t="n">
-        <v>0.03703703703703703</v>
+        <v>0.01587301587301587</v>
       </c>
       <c r="F59" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G59" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H59" s="7" t="n">
-        <v>-0.03703703703703703</v>
+        <v>0.05263157894736842</v>
+      </c>
+      <c r="H59" s="8" t="n">
+        <v>0.03675856307435255</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>10C2</t>
+          <t>12C1</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Geo</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Mlo</t>
+          <t>CBu</t>
         </is>
       </c>
       <c r="D60" s="4" t="n">
@@ -2383,17 +2383,17 @@
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>12C1</t>
+          <t>10C2</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>GL</t>
+          <t>Geo</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>CBu</t>
+          <t>Mlo</t>
         </is>
       </c>
       <c r="D61" s="4" t="n">
@@ -2464,7 +2464,7 @@
         <v>2</v>
       </c>
       <c r="E63" s="6" t="n">
-        <v>0.02439024390243903</v>
+        <v>0.02469135802469136</v>
       </c>
       <c r="F63" s="4" t="n">
         <v>4</v>
@@ -2473,39 +2473,39 @@
         <v>0.05882352941176471</v>
       </c>
       <c r="H63" s="8" t="n">
-        <v>0.03443328550932569</v>
+        <v>0.03413217138707335</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>11C1</t>
+          <t>10C2</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>CAl</t>
+          <t>Lza</t>
         </is>
       </c>
       <c r="D64" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E64" s="6" t="n">
-        <v>0</v>
+        <v>0.03389830508474576</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G64" s="6" t="n">
-        <v>0.03333333333333333</v>
-      </c>
-      <c r="H64" s="8" t="n">
-        <v>0.03333333333333333</v>
+        <v>0</v>
+      </c>
+      <c r="H64" s="7" t="n">
+        <v>-0.03389830508474576</v>
       </c>
     </row>
     <row r="65">
@@ -2543,33 +2543,33 @@
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>10C2</t>
+          <t>11C1</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Lza</t>
+          <t>CAl</t>
         </is>
       </c>
       <c r="D66" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E66" s="6" t="n">
-        <v>0.03278688524590164</v>
+        <v>0</v>
       </c>
       <c r="F66" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G66" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H66" s="7" t="n">
-        <v>-0.03278688524590164</v>
+        <v>0.03333333333333333</v>
+      </c>
+      <c r="H66" s="8" t="n">
+        <v>0.03333333333333333</v>
       </c>
     </row>
     <row r="67">
@@ -2592,7 +2592,7 @@
         <v>2</v>
       </c>
       <c r="E67" s="6" t="n">
-        <v>0.03125</v>
+        <v>0.03278688524590164</v>
       </c>
       <c r="F67" s="4" t="n">
         <v>0</v>
@@ -2601,45 +2601,45 @@
         <v>0</v>
       </c>
       <c r="H67" s="7" t="n">
-        <v>-0.03125</v>
+        <v>-0.03278688524590164</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>10C1</t>
+          <t>11C2</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Ing</t>
+          <t>Redação</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>APa</t>
+          <t>ACo</t>
         </is>
       </c>
       <c r="D68" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E68" s="6" t="n">
-        <v>0.06172839506172839</v>
+        <v>0.0975609756097561</v>
       </c>
       <c r="F68" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G68" s="6" t="n">
-        <v>0.09259259259259259</v>
-      </c>
-      <c r="H68" s="8" t="n">
-        <v>0.0308641975308642</v>
+        <v>0.06666666666666667</v>
+      </c>
+      <c r="H68" s="7" t="n">
+        <v>-0.03089430894308944</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>12C2</t>
+          <t>10C1</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
@@ -2649,61 +2649,61 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Isb</t>
+          <t>APa</t>
         </is>
       </c>
       <c r="D69" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E69" s="6" t="n">
-        <v>0.02272727272727273</v>
+        <v>0.06329113924050633</v>
       </c>
       <c r="F69" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G69" s="6" t="n">
-        <v>0.05263157894736842</v>
+        <v>0.09259259259259259</v>
       </c>
       <c r="H69" s="8" t="n">
-        <v>0.02990430622009569</v>
+        <v>0.02930145335208625</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>9C2</t>
+          <t>12C2</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>GL</t>
+          <t>Ing</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Caro</t>
+          <t>Isb</t>
         </is>
       </c>
       <c r="D70" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E70" s="6" t="n">
-        <v>0.01587301587301587</v>
+        <v>0.02380952380952381</v>
       </c>
       <c r="F70" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G70" s="6" t="n">
-        <v>0.04444444444444445</v>
+        <v>0.05263157894736842</v>
       </c>
       <c r="H70" s="8" t="n">
-        <v>0.02857142857142858</v>
+        <v>0.02882205513784461</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>9C1</t>
+          <t>9C2</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
@@ -2720,7 +2720,7 @@
         <v>1</v>
       </c>
       <c r="E71" s="6" t="n">
-        <v>0.01587301587301587</v>
+        <v>0.01612903225806452</v>
       </c>
       <c r="F71" s="4" t="n">
         <v>2</v>
@@ -2729,45 +2729,45 @@
         <v>0.04444444444444445</v>
       </c>
       <c r="H71" s="8" t="n">
-        <v>0.02857142857142858</v>
+        <v>0.02831541218637993</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>10C1</t>
+          <t>9C1</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Redação</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>BPad</t>
+          <t>Caro</t>
         </is>
       </c>
       <c r="D72" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E72" s="6" t="n">
-        <v>0.04878048780487805</v>
+        <v>0.01612903225806452</v>
       </c>
       <c r="F72" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G72" s="6" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.04444444444444445</v>
       </c>
       <c r="H72" s="8" t="n">
-        <v>0.02814258911819888</v>
+        <v>0.02831541218637993</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>9C1</t>
+          <t>9C2</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
@@ -2784,7 +2784,7 @@
         <v>2</v>
       </c>
       <c r="E73" s="6" t="n">
-        <v>0.01398601398601399</v>
+        <v>0.01428571428571429</v>
       </c>
       <c r="F73" s="4" t="n">
         <v>4</v>
@@ -2793,13 +2793,13 @@
         <v>0.04210526315789474</v>
       </c>
       <c r="H73" s="8" t="n">
-        <v>0.02811924917188075</v>
+        <v>0.02781954887218045</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>9C2</t>
+          <t>9C1</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
@@ -2816,7 +2816,7 @@
         <v>2</v>
       </c>
       <c r="E74" s="6" t="n">
-        <v>0.01398601398601399</v>
+        <v>0.01428571428571429</v>
       </c>
       <c r="F74" s="4" t="n">
         <v>4</v>
@@ -2825,71 +2825,71 @@
         <v>0.04210526315789474</v>
       </c>
       <c r="H74" s="8" t="n">
-        <v>0.02811924917188075</v>
+        <v>0.02781954887218045</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>11C1</t>
+          <t>10C1</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>DaF</t>
+          <t>Redação</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>CBu</t>
+          <t>BPad</t>
         </is>
       </c>
       <c r="D75" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E75" s="6" t="n">
-        <v>0.01204819277108434</v>
+        <v>0.05</v>
       </c>
       <c r="F75" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G75" s="6" t="n">
-        <v>0.03896103896103896</v>
+        <v>0.07692307692307693</v>
       </c>
       <c r="H75" s="8" t="n">
-        <v>0.02691284618995462</v>
+        <v>0.02692307692307692</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>11C2</t>
+          <t>11C1</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Redação</t>
+          <t>DaF</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>ACo</t>
+          <t>CBu</t>
         </is>
       </c>
       <c r="D76" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E76" s="6" t="n">
-        <v>0.09302325581395349</v>
+        <v>0.01234567901234568</v>
       </c>
       <c r="F76" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G76" s="6" t="n">
-        <v>0.06666666666666667</v>
-      </c>
-      <c r="H76" s="7" t="n">
-        <v>-0.02635658914728682</v>
+        <v>0.03896103896103896</v>
+      </c>
+      <c r="H76" s="8" t="n">
+        <v>0.02661535994869328</v>
       </c>
     </row>
     <row r="77">
@@ -2912,7 +2912,7 @@
         <v>2</v>
       </c>
       <c r="E77" s="6" t="n">
-        <v>0.02409638554216868</v>
+        <v>0.02469135802469136</v>
       </c>
       <c r="F77" s="4" t="n">
         <v>4</v>
@@ -2921,7 +2921,7 @@
         <v>0.05</v>
       </c>
       <c r="H77" s="8" t="n">
-        <v>0.02590361445783132</v>
+        <v>0.02530864197530864</v>
       </c>
     </row>
     <row r="78">
@@ -2959,97 +2959,97 @@
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>9C1</t>
+          <t>11C1</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>BrSa</t>
+          <t>Ale</t>
         </is>
       </c>
       <c r="D79" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E79" s="6" t="n">
-        <v>0.05714285714285714</v>
+        <v>0.0392156862745098</v>
       </c>
       <c r="F79" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G79" s="6" t="n">
-        <v>0.075</v>
-      </c>
-      <c r="H79" s="8" t="n">
-        <v>0.01785714285714286</v>
+        <v>0.02127659574468085</v>
+      </c>
+      <c r="H79" s="7" t="n">
+        <v>-0.01793909052982895</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>11C1</t>
+          <t>9C2</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Port</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Ale</t>
+          <t>Jana</t>
         </is>
       </c>
       <c r="D80" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E80" s="6" t="n">
-        <v>0.03883495145631068</v>
+        <v>0.04545454545454546</v>
       </c>
       <c r="F80" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G80" s="6" t="n">
-        <v>0.02127659574468085</v>
-      </c>
-      <c r="H80" s="7" t="n">
-        <v>-0.01755835571162983</v>
+        <v>0.0625</v>
+      </c>
+      <c r="H80" s="8" t="n">
+        <v>0.01704545454545454</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>9C2</t>
+          <t>9C1</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Port</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Jana</t>
+          <t>BrSa</t>
         </is>
       </c>
       <c r="D81" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E81" s="6" t="n">
-        <v>0.04545454545454546</v>
+        <v>0.05825242718446602</v>
       </c>
       <c r="F81" s="4" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G81" s="6" t="n">
-        <v>0.0625</v>
+        <v>0.075</v>
       </c>
       <c r="H81" s="8" t="n">
-        <v>0.01704545454545454</v>
+        <v>0.01674757281553398</v>
       </c>
     </row>
     <row r="82">
@@ -3072,7 +3072,7 @@
         <v>2</v>
       </c>
       <c r="E82" s="6" t="n">
-        <v>0.03333333333333333</v>
+        <v>0.03389830508474576</v>
       </c>
       <c r="F82" s="4" t="n">
         <v>3</v>
@@ -3081,71 +3081,71 @@
         <v>0.04838709677419355</v>
       </c>
       <c r="H82" s="8" t="n">
-        <v>0.01505376344086021</v>
+        <v>0.01448879168944778</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>9C1</t>
+          <t>11C2</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>Hist</t>
+          <t>DaF</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
         <is>
-          <t>JuLa</t>
+          <t>CBu</t>
         </is>
       </c>
       <c r="D83" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E83" s="6" t="n">
-        <v>0.04761904761904762</v>
+        <v>0.01234567901234568</v>
       </c>
       <c r="F83" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G83" s="6" t="n">
-        <v>0.0625</v>
+        <v>0.02597402597402598</v>
       </c>
       <c r="H83" s="8" t="n">
-        <v>0.01488095238095238</v>
+        <v>0.0136283469616803</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>11C2</t>
+          <t>9C1</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>DaF</t>
+          <t>Hist</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>CBu</t>
+          <t>JuLa</t>
         </is>
       </c>
       <c r="D84" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E84" s="6" t="n">
-        <v>0.01204819277108434</v>
+        <v>0.05</v>
       </c>
       <c r="F84" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G84" s="6" t="n">
-        <v>0.02597402597402598</v>
+        <v>0.0625</v>
       </c>
       <c r="H84" s="8" t="n">
-        <v>0.01392583320294164</v>
+        <v>0.0125</v>
       </c>
     </row>
     <row r="85">
@@ -3168,7 +3168,7 @@
         <v>2</v>
       </c>
       <c r="E85" s="6" t="n">
-        <v>0.03174603174603174</v>
+        <v>0.03225806451612903</v>
       </c>
       <c r="F85" s="4" t="n">
         <v>2</v>
@@ -3177,7 +3177,7 @@
         <v>0.04444444444444445</v>
       </c>
       <c r="H85" s="8" t="n">
-        <v>0.01269841269841272</v>
+        <v>0.01218637992831542</v>
       </c>
     </row>
     <row r="86">
@@ -3200,7 +3200,7 @@
         <v>2</v>
       </c>
       <c r="E86" s="6" t="n">
-        <v>0.03125</v>
+        <v>0.03225806451612903</v>
       </c>
       <c r="F86" s="4" t="n">
         <v>2</v>
@@ -3209,7 +3209,7 @@
         <v>0.04166666666666666</v>
       </c>
       <c r="H86" s="8" t="n">
-        <v>0.01041666666666666</v>
+        <v>0.009408602150537626</v>
       </c>
     </row>
     <row r="87">
@@ -3232,7 +3232,7 @@
         <v>1</v>
       </c>
       <c r="E87" s="6" t="n">
-        <v>0.01515151515151515</v>
+        <v>0.015625</v>
       </c>
       <c r="F87" s="4" t="n">
         <v>1</v>
@@ -3241,7 +3241,7 @@
         <v>0.025</v>
       </c>
       <c r="H87" s="8" t="n">
-        <v>0.009848484848484851</v>
+        <v>0.009375000000000001</v>
       </c>
     </row>
     <row r="88">
@@ -3264,7 +3264,7 @@
         <v>3</v>
       </c>
       <c r="E88" s="6" t="n">
-        <v>0.03488372093023256</v>
+        <v>0.03529411764705882</v>
       </c>
       <c r="F88" s="4" t="n">
         <v>3</v>
@@ -3273,7 +3273,7 @@
         <v>0.04411764705882353</v>
       </c>
       <c r="H88" s="8" t="n">
-        <v>0.009233926128590975</v>
+        <v>0.008823529411764709</v>
       </c>
     </row>
     <row r="89">
@@ -3296,7 +3296,7 @@
         <v>4</v>
       </c>
       <c r="E89" s="6" t="n">
-        <v>0.0396039603960396</v>
+        <v>0.04</v>
       </c>
       <c r="F89" s="4" t="n">
         <v>2</v>
@@ -3305,23 +3305,23 @@
         <v>0.04444444444444445</v>
       </c>
       <c r="H89" s="9" t="n">
-        <v>0.004840484048404856</v>
+        <v>0.004444444444444452</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>12C1</t>
+          <t>9C1</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Geo</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>Fab</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D90" s="4" t="n">
@@ -3334,42 +3334,42 @@
         <v>2</v>
       </c>
       <c r="G90" s="6" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.06666666666666667</v>
       </c>
       <c r="H90" s="9" t="n">
-        <v>0.001661129568106309</v>
+        <v>-0.00310077519379845</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>9C1</t>
+          <t>12C1</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>Geo</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Fab</t>
         </is>
       </c>
       <c r="D91" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E91" s="6" t="n">
-        <v>0.06818181818181818</v>
+        <v>0.06976744186046512</v>
       </c>
       <c r="F91" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G91" s="6" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.07142857142857142</v>
       </c>
       <c r="H91" s="9" t="n">
-        <v>-0.001515151515151511</v>
+        <v>0.001661129568106309</v>
       </c>
     </row>
     <row r="92">
@@ -3380,89 +3380,89 @@
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Geo</t>
+          <t>Hist</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>Mar</t>
+          <t>Wag</t>
         </is>
       </c>
       <c r="D92" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E92" s="6" t="n">
-        <v>0.04878048780487805</v>
+        <v>0.02439024390243903</v>
       </c>
       <c r="F92" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G92" s="6" t="n">
-        <v>0.05</v>
+        <v>0.02380952380952381</v>
       </c>
       <c r="H92" s="9" t="n">
-        <v>0.001219512195121952</v>
+        <v>-0.000580720092915217</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>12C2</t>
+          <t>12C1</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>Hist</t>
+          <t>Redação</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
         <is>
-          <t>Wag</t>
+          <t>AMu</t>
         </is>
       </c>
       <c r="D93" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E93" s="6" t="n">
-        <v>0.02439024390243903</v>
+        <v>0.07142857142857142</v>
       </c>
       <c r="F93" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G93" s="6" t="n">
-        <v>0.02380952380952381</v>
+        <v>0.07142857142857142</v>
       </c>
       <c r="H93" s="9" t="n">
-        <v>-0.000580720092915217</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>12C1</t>
+          <t>12C2</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>Redação</t>
+          <t>Geo</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>AMu</t>
+          <t>Mar</t>
         </is>
       </c>
       <c r="D94" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E94" s="6" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.05</v>
       </c>
       <c r="F94" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G94" s="6" t="n">
-        <v>0.07142857142857142</v>
+        <v>0.05</v>
       </c>
       <c r="H94" s="9" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Confirma a leitura da prova de Sociologia da 12C1 e as interpretações
A escola confirmou que a célula incompleta da 12C1 (semana 16, quarta,
3º tempo) é Sociologia. Entra em CORRECOES, mecanismo para leituras que a
escola valida a mão quando o arquivo está incompleto e a turma irmã não
serve de referência — aqui não servia, porque na 12C2 a Sociologia caiu
no 6º tempo.

A prova caiu no próprio tempo de Sociologia da 12C1 (quarta, 3º, prof.
Kle), então não gera cessão e os totais não mudam. De quebra, é uma
conferência cruzada da grade extraída do PDF: o calendário e a grade
concordam sobre onde fica a aula de Sociologia.

As cinco decisões de interpretação também foram confirmadas e passam de
'em aberto' para 'validadas' na referência. Restam só as duas células
ilegíveis da 10C1.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4DDeWeQcpRs26bquKMMCA
</commit_message>
<xml_diff>
--- a/Horario desenvolvido/Comparativo_Cessoes_1SEM_x_Proposta3.xlsx
+++ b/Horario desenvolvido/Comparativo_Cessoes_1SEM_x_Proposta3.xlsx
@@ -847,7 +847,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>10C2</t>
+          <t>10C1</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -879,7 +879,7 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>10C1</t>
+          <t>10C2</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -980,12 +980,12 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Port</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>FBri</t>
+          <t>MFo</t>
         </is>
       </c>
       <c r="D17" s="4" t="n">
@@ -1012,12 +1012,12 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Port</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>MFo</t>
+          <t>FBri</t>
         </is>
       </c>
       <c r="D18" s="4" t="n">
@@ -1103,17 +1103,17 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>12C2</t>
+          <t>10C1</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Fis</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Cadu</t>
+          <t>CAl</t>
         </is>
       </c>
       <c r="D21" s="4" t="n">
@@ -1135,7 +1135,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>12C1</t>
+          <t>10C2</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -1145,29 +1145,29 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Wag</t>
+          <t>ALu</t>
         </is>
       </c>
       <c r="D22" s="4" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="6" t="n">
         <v>0.07142857142857142</v>
       </c>
-      <c r="F22" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" s="7" t="n">
-        <v>-0.07142857142857142</v>
+      <c r="H22" s="8" t="n">
+        <v>0.07142857142857142</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>10C2</t>
+          <t>12C1</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -1177,39 +1177,39 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>ALu</t>
+          <t>Wag</t>
         </is>
       </c>
       <c r="D23" s="4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>0</v>
+        <v>0.07142857142857142</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>0.07142857142857142</v>
-      </c>
-      <c r="H23" s="8" t="n">
-        <v>0.07142857142857142</v>
+        <v>0</v>
+      </c>
+      <c r="H23" s="7" t="n">
+        <v>-0.07142857142857142</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>10C1</t>
+          <t>12C2</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Fis</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>CAl</t>
+          <t>Cadu</t>
         </is>
       </c>
       <c r="D24" s="4" t="n">
@@ -1359,17 +1359,17 @@
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>9C1</t>
+          <t>11C2</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Port</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Jana</t>
+          <t>JJ</t>
         </is>
       </c>
       <c r="D29" s="4" t="n">
@@ -1391,17 +1391,17 @@
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>11C1</t>
+          <t>11C2</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>JJ</t>
+          <t>CAl</t>
         </is>
       </c>
       <c r="D30" s="4" t="n">
@@ -1423,7 +1423,7 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>11C2</t>
+          <t>11C1</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
@@ -1455,17 +1455,17 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>11C2</t>
+          <t>9C1</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Port</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>CAl</t>
+          <t>Jana</t>
         </is>
       </c>
       <c r="D32" s="4" t="n">
@@ -1583,17 +1583,17 @@
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>12C2</t>
+          <t>11C2</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Bio</t>
+          <t>Ing</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Ale</t>
+          <t>PaH</t>
         </is>
       </c>
       <c r="D36" s="4" t="n">
@@ -1603,7 +1603,7 @@
         <v>0</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G36" s="6" t="n">
         <v>0.05</v>
@@ -1615,39 +1615,39 @@
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>11C2</t>
+          <t>10C1</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Ing</t>
+          <t>Bio</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>PaH</t>
+          <t>Lza</t>
         </is>
       </c>
       <c r="D37" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E37" s="6" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G37" s="6" t="n">
         <v>0.05</v>
       </c>
-      <c r="H37" s="8" t="n">
-        <v>0.05</v>
+      <c r="H37" s="7" t="n">
+        <v>-0.05</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>10C1</t>
+          <t>12C2</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
@@ -1657,14 +1657,14 @@
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Lza</t>
+          <t>Ale</t>
         </is>
       </c>
       <c r="D38" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E38" s="6" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="F38" s="4" t="n">
         <v>2</v>
@@ -1672,8 +1672,8 @@
       <c r="G38" s="6" t="n">
         <v>0.05</v>
       </c>
-      <c r="H38" s="7" t="n">
-        <v>-0.05</v>
+      <c r="H38" s="8" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="39">
@@ -1871,21 +1871,21 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>12C1</t>
+          <t>11C2</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Fil</t>
+          <t>Hist</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>LAn</t>
+          <t>Ver</t>
         </is>
       </c>
       <c r="D45" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E45" s="6" t="n">
         <v>0.04761904761904762</v>
@@ -1903,39 +1903,39 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>10C2</t>
+          <t>12C1</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>Mat</t>
+          <t>Fil</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>BrSa</t>
+          <t>LAn</t>
         </is>
       </c>
       <c r="D46" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E46" s="6" t="n">
-        <v>0</v>
+        <v>0.04761904761904762</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G46" s="6" t="n">
-        <v>0.04761904761904762</v>
-      </c>
-      <c r="H46" s="8" t="n">
-        <v>0.04761904761904762</v>
+        <v>0</v>
+      </c>
+      <c r="H46" s="7" t="n">
+        <v>-0.04761904761904762</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>10C1</t>
+          <t>10C2</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -1967,33 +1967,33 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>11C2</t>
+          <t>10C1</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Hist</t>
+          <t>Mat</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Ver</t>
+          <t>BrSa</t>
         </is>
       </c>
       <c r="D48" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G48" s="6" t="n">
         <v>0.04761904761904762</v>
       </c>
-      <c r="F48" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" s="7" t="n">
-        <v>-0.04761904761904762</v>
+      <c r="H48" s="8" t="n">
+        <v>0.04761904761904762</v>
       </c>
     </row>
     <row r="49">
@@ -2255,7 +2255,7 @@
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>9C2</t>
+          <t>9C1</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
@@ -2287,7 +2287,7 @@
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>9C1</t>
+          <t>9C2</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
@@ -2351,7 +2351,7 @@
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>12C1</t>
+          <t>12C2</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
@@ -2383,17 +2383,17 @@
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>10C2</t>
+          <t>12C1</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Geo</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Mlo</t>
+          <t>CBu</t>
         </is>
       </c>
       <c r="D61" s="4" t="n">
@@ -2415,17 +2415,17 @@
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>12C2</t>
+          <t>10C2</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>GL</t>
+          <t>Geo</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>CBu</t>
+          <t>Mlo</t>
         </is>
       </c>
       <c r="D62" s="4" t="n">
@@ -2516,12 +2516,12 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>GL</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>CBu</t>
+          <t>CAl</t>
         </is>
       </c>
       <c r="D65" s="4" t="n">
@@ -2548,12 +2548,12 @@
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>GL</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>CAl</t>
+          <t>CBu</t>
         </is>
       </c>
       <c r="D66" s="4" t="n">
@@ -2703,7 +2703,7 @@
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>9C2</t>
+          <t>9C1</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
@@ -2735,7 +2735,7 @@
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>9C1</t>
+          <t>9C2</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">

</xml_diff>